<commit_message>
Updated Cell referencing and Formulation
</commit_message>
<xml_diff>
--- a/Excel Practice @ Day 01.xlsx
+++ b/Excel Practice @ Day 01.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\26-Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0F78FD-AF34-4B06-9BC0-1F431753CC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19200" windowHeight="7510"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,11 +14,24 @@
     <definedName name="Basic_Salary">Sheet2!$I$2:$I$39</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="141">
   <si>
     <t>Product</t>
   </si>
@@ -95,7 +102,19 @@
     <t>A18*D17</t>
   </si>
   <si>
+    <t>A18*E17</t>
+  </si>
+  <si>
+    <t>A18*F17</t>
+  </si>
+  <si>
     <t>A19*B17</t>
+  </si>
+  <si>
+    <t>A18*C19</t>
+  </si>
+  <si>
+    <t>A19*D17</t>
   </si>
   <si>
     <t>A20*B17</t>
@@ -440,12 +459,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="&quot;₹&quot;#,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;₹&quot;\ #,##0.00"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="7">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="dd/mmm/yy"/>
+    <numFmt numFmtId="181" formatCode="&quot;₹&quot;#,##0"/>
+    <numFmt numFmtId="182" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -473,28 +497,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -506,8 +510,152 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -526,8 +674,194 @@
         <bgColor rgb="FFA8D08D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -576,25 +910,270 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -603,41 +1182,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="182" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="166" formatCode="&quot;₹&quot;#,##0"/>
+      <numFmt numFmtId="180" formatCode="dd/mmm/yy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="20" formatCode="dd/mmm/yy"/>
+      <numFmt numFmtId="181" formatCode="&quot;₹&quot;#,##0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -645,26 +1265,23 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I39" totalsRowShown="0">
-  <autoFilter ref="A1:I39" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I39" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I39" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="C_Code"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Birthdate" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Gender"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="M_Status"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Department"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Region"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Basic Salary" dataDxfId="0"/>
+    <tableColumn id="1" name="C_Code"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Birthdate" dataDxfId="0"/>
+    <tableColumn id="5" name="Gender"/>
+    <tableColumn id="6" name="M_Status"/>
+    <tableColumn id="7" name="Department"/>
+    <tableColumn id="8" name="Region"/>
+    <tableColumn id="9" name="Basic Salary" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -922,105 +1539,107 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A2:N25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="5" max="5" width="12.1796875" customWidth="1"/>
+    <col min="5" max="5" width="12.1818181818182" customWidth="1"/>
+    <col min="12" max="12" width="10"/>
+    <col min="14" max="14" width="10.1818181818182"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" ht="29">
-      <c r="A2" s="9" t="s">
+    <row r="2" ht="29" spans="1:14">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="11">
         <v>40000</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="11">
         <v>2</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="11">
         <f>B3*C3</f>
         <v>80000</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <f>D3/$D$6</f>
-        <v>0.83333333333333304</v>
-      </c>
-      <c r="K3" s="12" t="s">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="K3" s="13" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="11">
         <v>2000</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="11">
         <v>5</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <f>B4*C4</f>
         <v>10000</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <f>D4/$D$6</f>
         <v>0.104166666666667</v>
       </c>
-      <c r="J4" s="12"/>
-      <c r="K4" s="13">
+      <c r="J4" s="13"/>
+      <c r="K4" s="14">
         <v>0.4</v>
       </c>
-      <c r="L4" s="13">
+      <c r="L4" s="14">
         <v>1.2</v>
       </c>
-      <c r="M4" s="13">
+      <c r="M4" s="14">
         <v>0.12</v>
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="11">
         <v>2000</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="11">
         <v>3</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>B5*C5</f>
         <v>6000</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <f>D5/$D$6</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="J5" s="12" t="s">
+        <v>0.0625</v>
+      </c>
+      <c r="J5" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K5" t="s">
@@ -1065,17 +1684,17 @@
         <v>314</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="27" customHeight="1">
-      <c r="A8" s="9" t="s">
+    <row r="8" ht="27" customHeight="1" spans="1:14">
+      <c r="A8" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>14</v>
       </c>
       <c r="J8" t="s">
@@ -1092,16 +1711,16 @@
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="11">
         <v>50000</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="15">
         <v>0.1</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="11">
         <f>B9*$C$9</f>
         <v>5000</v>
       </c>
@@ -1119,14 +1738,14 @@
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="11">
         <v>1000</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="10">
+      <c r="C10" s="15"/>
+      <c r="D10" s="11">
         <f t="shared" ref="D10:D11" si="0">B10*$C$9</f>
         <v>100</v>
       </c>
@@ -1144,14 +1763,14 @@
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="11">
         <v>2000</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="10">
+      <c r="C11" s="15"/>
+      <c r="D11" s="11">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
@@ -1169,10 +1788,10 @@
       </c>
     </row>
     <row r="13" spans="1:14">
-      <c r="B13" s="15"/>
+      <c r="B13" s="16"/>
     </row>
     <row r="14" spans="1:14">
-      <c r="J14" s="12" t="s">
+      <c r="J14" s="13" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1191,130 +1810,286 @@
       </c>
     </row>
     <row r="16" spans="1:14">
-      <c r="B16" s="9"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
       <c r="J16" t="s">
         <v>11</v>
       </c>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="17"/>
+      <c r="K16" s="14">
+        <f>K6*$K$4</f>
+        <v>145.6</v>
+      </c>
+      <c r="L16" s="14">
+        <f>L6*$L$4</f>
+        <v>469.2</v>
+      </c>
+      <c r="M16" s="14">
+        <f>M6*$M$4</f>
+        <v>26.4</v>
+      </c>
+      <c r="N16" s="18">
+        <f>SUM(K16:M16)</f>
+        <v>641.2</v>
+      </c>
     </row>
     <row r="17" spans="1:14">
       <c r="B17">
         <v>1</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>2</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>3</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="16">
         <v>4</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="16">
         <v>5</v>
       </c>
       <c r="J17" t="s">
         <v>12</v>
       </c>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="17"/>
+      <c r="K17" s="14">
+        <f>K7*$K$4</f>
+        <v>154.8</v>
+      </c>
+      <c r="L17" s="14">
+        <f>L7*$L$4</f>
+        <v>294</v>
+      </c>
+      <c r="M17" s="14">
+        <f>M7*$M$4</f>
+        <v>37.68</v>
+      </c>
+      <c r="N17" s="18">
+        <f>SUM(K17:M17)</f>
+        <v>486.48</v>
+      </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="18">
+      <c r="A18" s="19">
         <v>1</v>
       </c>
-      <c r="B18" s="15">
-        <f>A18*B17</f>
+      <c r="B18" s="16">
+        <f>$A18*B$17</f>
         <v>1</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="C18" s="16">
+        <f>$A18*C$17</f>
+        <v>2</v>
+      </c>
+      <c r="D18" s="16">
+        <f>$A18*D$17</f>
+        <v>3</v>
+      </c>
+      <c r="E18" s="16">
+        <f>$A18*E$17</f>
+        <v>4</v>
+      </c>
+      <c r="F18" s="16">
+        <f>$A18*F$17</f>
+        <v>5</v>
+      </c>
       <c r="J18" t="s">
         <v>15</v>
       </c>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="17"/>
+      <c r="K18" s="14">
+        <f>K8*$K$4</f>
+        <v>116</v>
+      </c>
+      <c r="L18" s="14">
+        <f>L8*$L$4</f>
+        <v>253.2</v>
+      </c>
+      <c r="M18" s="14">
+        <f>M8*$M$4</f>
+        <v>24</v>
+      </c>
+      <c r="N18" s="18">
+        <f>SUM(K18:M18)</f>
+        <v>393.2</v>
+      </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="18">
+      <c r="A19" s="19">
         <v>2</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+      <c r="B19" s="16">
+        <f>A19*$B$17</f>
+        <v>2</v>
+      </c>
+      <c r="C19" s="16">
+        <f>$A19*C$17</f>
+        <v>4</v>
+      </c>
+      <c r="D19" s="16">
+        <f>$A19*D$17</f>
+        <v>6</v>
+      </c>
+      <c r="E19" s="16">
+        <f>$A19*E$17</f>
+        <v>8</v>
+      </c>
+      <c r="F19" s="16">
+        <f>$A19*F$17</f>
+        <v>10</v>
+      </c>
       <c r="J19" t="s">
         <v>16</v>
       </c>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="17"/>
+      <c r="K19" s="14">
+        <f>K9*$K$4</f>
+        <v>136</v>
+      </c>
+      <c r="L19" s="14">
+        <f>L9*$L$4</f>
+        <v>318</v>
+      </c>
+      <c r="M19" s="14">
+        <f>M9*$M$4</f>
+        <v>39.6</v>
+      </c>
+      <c r="N19" s="18">
+        <f>SUM(K19:M19)</f>
+        <v>493.6</v>
+      </c>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="18">
+      <c r="A20" s="19">
         <v>3</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
+      <c r="B20" s="16">
+        <f>A20*$B$17</f>
+        <v>3</v>
+      </c>
+      <c r="C20" s="16">
+        <f>$A20*C$17</f>
+        <v>6</v>
+      </c>
+      <c r="D20" s="16">
+        <f>$A20*D$17</f>
+        <v>9</v>
+      </c>
+      <c r="E20" s="16">
+        <f>$A20*E$17</f>
+        <v>12</v>
+      </c>
+      <c r="F20" s="16">
+        <f>$A20*F$17</f>
+        <v>15</v>
+      </c>
       <c r="J20" t="s">
         <v>17</v>
       </c>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="17"/>
+      <c r="K20" s="14">
+        <f>K10*$K$4</f>
+        <v>104.4</v>
+      </c>
+      <c r="L20" s="14">
+        <f>L10*$L$4</f>
+        <v>414</v>
+      </c>
+      <c r="M20" s="14">
+        <f>M10*$M$4</f>
+        <v>29.52</v>
+      </c>
+      <c r="N20" s="18">
+        <f>SUM(K20:M20)</f>
+        <v>547.92</v>
+      </c>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="18">
+      <c r="A21" s="19">
         <v>4</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="B21" s="16">
+        <f>A21*$B$17</f>
+        <v>4</v>
+      </c>
+      <c r="C21" s="16">
+        <f>$A21*C$17</f>
+        <v>8</v>
+      </c>
+      <c r="D21" s="16">
+        <f>$A21*D$17</f>
+        <v>12</v>
+      </c>
+      <c r="E21" s="16">
+        <f>$A21*E$17</f>
+        <v>16</v>
+      </c>
+      <c r="F21" s="16">
+        <f>$A21*F$17</f>
+        <v>20</v>
+      </c>
       <c r="J21" t="s">
         <v>18</v>
       </c>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="17"/>
+      <c r="K21" s="14">
+        <f>K11*$K$4</f>
+        <v>146</v>
+      </c>
+      <c r="L21" s="14">
+        <f>L11*$L$4</f>
+        <v>278.4</v>
+      </c>
+      <c r="M21" s="14">
+        <f>M11*$M$4</f>
+        <v>46.8</v>
+      </c>
+      <c r="N21" s="18">
+        <f>SUM(K21:M21)</f>
+        <v>471.2</v>
+      </c>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="18">
+      <c r="A22" s="19">
         <v>5</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="J22" s="12" t="s">
+      <c r="B22" s="16">
+        <f>A22*$B$17</f>
+        <v>5</v>
+      </c>
+      <c r="C22" s="16">
+        <f>$A22*C$17</f>
+        <v>10</v>
+      </c>
+      <c r="D22" s="16">
+        <f>$A22*D$17</f>
+        <v>15</v>
+      </c>
+      <c r="E22" s="16">
+        <f>$A22*E$17</f>
+        <v>20</v>
+      </c>
+      <c r="F22" s="16">
+        <f>$A22*F$17</f>
+        <v>25</v>
+      </c>
+      <c r="J22" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="17"/>
+      <c r="K22" s="14">
+        <f>SUM(K16:K21)</f>
+        <v>802.8</v>
+      </c>
+      <c r="L22" s="14">
+        <f>SUM(L16:L21)</f>
+        <v>2026.8</v>
+      </c>
+      <c r="M22" s="14">
+        <f>SUM(M16:M21)</f>
+        <v>204</v>
+      </c>
+      <c r="N22" s="18">
+        <f>SUM(K22:M22)</f>
+        <v>3033.6</v>
+      </c>
     </row>
     <row r="23" spans="1:14">
       <c r="B23" t="s">
@@ -1326,69 +2101,83 @@
       <c r="D23" t="s">
         <v>22</v>
       </c>
+      <c r="E23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="24" spans="1:14">
       <c r="B24" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:14">
       <c r="B25" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:P39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.36328125" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" customWidth="1"/>
-    <col min="3" max="3" width="11.1796875" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" customWidth="1"/>
+    <col min="1" max="1" width="9.36363636363636" customWidth="1"/>
+    <col min="2" max="2" width="11.3636363636364" customWidth="1"/>
+    <col min="3" max="3" width="11.1818181818182" customWidth="1"/>
+    <col min="4" max="4" width="10.6363636363636" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" customWidth="1"/>
+    <col min="6" max="6" width="10.9090909090909" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12.6328125" customWidth="1"/>
-    <col min="12" max="12" width="48.6328125" customWidth="1"/>
-    <col min="13" max="13" width="13.08984375" customWidth="1"/>
-    <col min="14" max="14" width="11.6328125" customWidth="1"/>
-    <col min="15" max="15" width="13.453125" customWidth="1"/>
+    <col min="9" max="9" width="12.6363636363636" customWidth="1"/>
+    <col min="12" max="12" width="48.6363636363636" customWidth="1"/>
+    <col min="13" max="13" width="13.0909090909091" customWidth="1"/>
+    <col min="14" max="14" width="11.6363636363636" customWidth="1"/>
+    <col min="15" max="15" width="13.4545454545455" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -1396,25 +2185,25 @@
         <v>150834</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D2" s="2">
         <v>31199</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I2" s="3">
         <v>48000</v>
@@ -1425,25 +2214,25 @@
         <v>150784</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D3" s="2">
         <v>28365</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" t="s">
         <v>43</v>
-      </c>
-      <c r="H3" t="s">
-        <v>39</v>
       </c>
       <c r="I3" s="3">
         <v>35000</v>
@@ -1454,256 +2243,256 @@
         <v>150791</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D4" s="2">
         <v>59871</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
         <v>43</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
       </c>
       <c r="I4" s="3">
         <v>67000</v>
       </c>
-      <c r="L4" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" s="21"/>
+      <c r="L4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5"/>
     </row>
     <row r="5" spans="1:13">
       <c r="A5">
         <v>150940</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D5" s="2">
         <v>26906</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I5" s="3">
         <v>87000</v>
       </c>
-      <c r="L5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="M5" s="5"/>
+      <c r="L5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="7"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6">
         <v>150777</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D6" s="2">
         <v>57648</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I6" s="3">
         <v>22000</v>
       </c>
-      <c r="L6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" s="5"/>
+      <c r="L6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M6" s="7"/>
     </row>
     <row r="7" spans="1:13">
       <c r="A7">
         <v>150805</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2">
         <v>26172</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3">
         <v>91000</v>
       </c>
-      <c r="L7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M7" s="6"/>
+      <c r="L7" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M7" s="8"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8">
         <v>150990</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D8" s="2">
         <v>36400</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I8" s="3">
         <v>77000</v>
       </c>
-      <c r="L8" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="M8" s="6"/>
+      <c r="L8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="8"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9">
         <v>150989</v>
       </c>
       <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" t="s">
         <v>65</v>
-      </c>
-      <c r="C9" t="s">
-        <v>61</v>
       </c>
       <c r="D9" s="2">
         <v>33113</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I9" s="3">
         <v>45000</v>
       </c>
-      <c r="L9" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="M9" s="6"/>
+      <c r="L9" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M9" s="8"/>
     </row>
     <row r="10" spans="1:13">
       <c r="A10">
         <v>150881</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D10" s="2">
         <v>30337</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I10" s="3">
         <v>92000</v>
       </c>
-      <c r="L10" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="M10" s="6"/>
+      <c r="L10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M10" s="8"/>
     </row>
     <row r="11" spans="1:13">
       <c r="A11">
         <v>150814</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D11" s="2">
         <v>26246</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I11" s="3">
         <v>50000</v>
@@ -1714,256 +2503,256 @@
         <v>150937</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2">
         <v>61225</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I12" s="3">
         <v>37000</v>
       </c>
-      <c r="L12" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="M12" s="21"/>
+      <c r="L12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="M12" s="5"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13">
         <v>150888</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D13" s="2">
         <v>29221</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F13" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I13" s="3">
         <v>43000</v>
       </c>
-      <c r="L13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="M13" s="6"/>
+      <c r="L13" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="M13" s="8"/>
     </row>
     <row r="14" spans="1:13">
       <c r="A14">
         <v>150865</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D14" s="2">
         <v>31279</v>
       </c>
       <c r="E14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I14" s="3">
         <v>90000</v>
       </c>
-      <c r="L14" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="M14" s="6"/>
+      <c r="L14" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="M14" s="8"/>
     </row>
     <row r="15" spans="1:13">
       <c r="A15">
         <v>150858</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D15" s="2">
         <v>34846</v>
       </c>
       <c r="E15" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I15" s="3">
         <v>34000</v>
       </c>
-      <c r="L15" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="M15" s="6"/>
+      <c r="L15" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="M15" s="8"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16">
         <v>150930</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D16" s="2">
         <v>37027</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F16" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G16" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I16" s="3">
         <v>82000</v>
       </c>
-      <c r="L16" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="M16" s="6"/>
+      <c r="L16" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M16" s="8"/>
     </row>
     <row r="17" spans="1:16">
       <c r="A17">
         <v>150894</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D17" s="2">
         <v>37124</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H17" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I17" s="3">
         <v>67000</v>
       </c>
-      <c r="L17" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="M17" s="6"/>
+      <c r="L17" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="M17" s="8"/>
     </row>
     <row r="18" spans="1:16">
       <c r="A18">
         <v>150947</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C18" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D18" s="2">
         <v>33449</v>
       </c>
       <c r="E18" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H18" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I18" s="3">
         <v>85000</v>
       </c>
-      <c r="L18" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="M18" s="6"/>
+      <c r="L18" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M18" s="8"/>
     </row>
     <row r="19" spans="1:16">
       <c r="A19">
         <v>150905</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D19" s="2">
         <v>30819</v>
       </c>
       <c r="E19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F19" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="G19" t="s">
-        <v>38</v>
-      </c>
       <c r="H19" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I19" s="3">
         <v>62000</v>
@@ -1974,25 +2763,25 @@
         <v>150995</v>
       </c>
       <c r="B20" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D20" s="2">
         <v>35330</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G20" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I20" s="3">
         <v>15000</v>
@@ -2003,25 +2792,25 @@
         <v>150912</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D21" s="2">
         <v>37629</v>
       </c>
       <c r="E21" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F21" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G21" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H21" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I21" s="3">
         <v>81000</v>
@@ -2032,76 +2821,76 @@
         <v>150921</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D22" s="2">
         <v>38092</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F22" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G22" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H22" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I22" s="3">
         <v>19000</v>
       </c>
-      <c r="L22" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="M22" s="21"/>
+      <c r="L22" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="M22" s="5"/>
     </row>
     <row r="23" spans="1:16">
       <c r="A23">
         <v>150851</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C23" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D23" s="2">
         <v>29368</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F23" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G23" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H23" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I23" s="3">
         <v>75000</v>
       </c>
-      <c r="L23" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N23" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="O23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="P23" s="4" t="s">
-        <v>63</v>
+      <c r="L23" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="O23" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -2109,421 +2898,421 @@
         <v>150867</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D24" s="2">
         <v>29028</v>
       </c>
       <c r="E24" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G24" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H24" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I24" s="3">
         <v>49000</v>
       </c>
-      <c r="L24" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
+      <c r="L24" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
     </row>
     <row r="25" spans="1:16">
       <c r="A25">
         <v>150899</v>
       </c>
       <c r="B25" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D25" s="2">
         <v>37400</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F25" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H25" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I25" s="3">
         <v>50000</v>
       </c>
-      <c r="L25" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
+      <c r="L25" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
     </row>
     <row r="26" spans="1:16">
       <c r="A26">
         <v>150975</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D26" s="2">
         <v>31478</v>
       </c>
       <c r="E26" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F26" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I26" s="3">
         <v>83000</v>
       </c>
-      <c r="L26" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
+      <c r="L26" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
     </row>
     <row r="27" spans="1:16">
       <c r="A27">
         <v>150901</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D27" s="2">
         <v>32946</v>
       </c>
       <c r="E27" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F27" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G27" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H27" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I27" s="3">
         <v>53000</v>
       </c>
-      <c r="L27" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="M27" s="6"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="6"/>
-      <c r="P27" s="6"/>
+      <c r="L27" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
     </row>
     <row r="28" spans="1:16">
       <c r="A28">
         <v>150968</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C28" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D28" s="2">
         <v>37208</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F28" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G28" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H28" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I28" s="3">
         <v>65000</v>
       </c>
-      <c r="L28" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="M28" s="6"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
+      <c r="L28" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29">
         <v>150773</v>
       </c>
       <c r="B29" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D29" s="2">
         <v>26860</v>
       </c>
       <c r="E29" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F29" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G29" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H29" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I29" s="3">
         <v>85000</v>
       </c>
-      <c r="L29" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
+      <c r="L29" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
     </row>
     <row r="30" spans="1:16">
       <c r="A30">
         <v>150840</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D30" s="2">
         <v>59661</v>
       </c>
       <c r="E30" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F30" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G30" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H30" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I30" s="3">
         <v>20000</v>
       </c>
-      <c r="L30" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
+      <c r="L30" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
     </row>
     <row r="31" spans="1:16">
       <c r="A31">
         <v>150850</v>
       </c>
       <c r="B31" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D31" s="2">
         <v>32027</v>
       </c>
       <c r="E31" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F31" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G31" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H31" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I31" s="3">
         <v>47000</v>
       </c>
-      <c r="L31" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
+      <c r="L31" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
     </row>
     <row r="32" spans="1:16">
       <c r="A32">
         <v>150962</v>
       </c>
       <c r="B32" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D32" s="2">
         <v>37773</v>
       </c>
       <c r="E32" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F32" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G32" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H32" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I32" s="3">
         <v>87000</v>
       </c>
-      <c r="L32" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
+      <c r="L32" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
     </row>
     <row r="33" spans="1:16">
       <c r="A33">
         <v>150954</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D33" s="2">
         <v>35495</v>
       </c>
       <c r="E33" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F33" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G33" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H33" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I33" s="3">
         <v>57000</v>
       </c>
-      <c r="L33" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6"/>
-      <c r="P33" s="6"/>
+      <c r="L33" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
     </row>
     <row r="34" spans="1:16">
       <c r="A34">
         <v>150874</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C34" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D34" s="2">
         <v>37890</v>
       </c>
       <c r="E34" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F34" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G34" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I34" s="3">
         <v>27000</v>
       </c>
-      <c r="L34" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="M34" s="6"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="6"/>
-      <c r="P34" s="6"/>
+      <c r="L34" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
     </row>
     <row r="35" spans="1:16">
       <c r="A35">
         <v>150798</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C35" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D35" s="2">
         <v>28276</v>
       </c>
       <c r="E35" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F35" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G35" t="s">
+        <v>47</v>
+      </c>
+      <c r="H35" t="s">
         <v>43</v>
-      </c>
-      <c r="H35" t="s">
-        <v>39</v>
       </c>
       <c r="I35" s="3">
         <v>81000</v>
@@ -2534,25 +3323,25 @@
         <v>150830</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D36" s="2">
         <v>29037</v>
       </c>
       <c r="E36" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F36" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G36" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H36" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I36" s="3">
         <v>52000</v>
@@ -2563,25 +3352,25 @@
         <v>150929</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C37" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D37" s="2">
         <v>26739</v>
       </c>
       <c r="E37" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F37" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H37" t="s">
         <v>55</v>
-      </c>
-      <c r="H37" t="s">
-        <v>51</v>
       </c>
       <c r="I37" s="3">
         <v>58000</v>
@@ -2592,25 +3381,25 @@
         <v>150982</v>
       </c>
       <c r="B38" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D38" s="2">
         <v>35574</v>
       </c>
       <c r="E38" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F38" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G38" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H38" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I38" s="3">
         <v>47000</v>
@@ -2621,25 +3410,25 @@
         <v>150821</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D39" s="2">
         <v>29966</v>
       </c>
       <c r="E39" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F39" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G39" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H39" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I39" s="3">
         <v>26000</v>
@@ -2652,6 +3441,7 @@
     <mergeCell ref="L22:M22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2659,11 +3449,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<DataMashup xmlns="http://schemas.microsoft.com/DataMashup">AAAAAGwDAABQSwMECgAAAAAAh07iQAAAAAAAAAAAAAAAAAcAAABDb25maWcvUEsDBBQAAAAIAIdO4kASOP6YnwAAAPMAAAASAAAAQ29uZmlnL1BhY2thZ2UueG1shY9NC4IwHMa/iuzuNmdRyN958JoRBNF1zDVHOsPNJn36jDK6dXtefofngWLq2uiuBmd6m6MEUxQpK/vaWJ2j0V/iLSo4HIS8Cq2iGbYum1ydo8b7W0ZICAGHFPeDJozShJyr3VE2qhPoC5v/cGys88JKhTic3mM4w8lqg9N1iimQJYTK2EUzzOa9r/YnhHJs/Tgo/mjicg9ksUA+H/gTUEsDBAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAARm9ybXVsYXMvUEsDBBQAAAAIAIdO4kAoike4DgAAABEAAAATAAAARm9ybXVsYXMvU2VjdGlvbjEubStOTS7JzM9TCIbQhtYAUEsDBBQAAAAIAIdO4kB/v9PKnQAAAOQAAAATAAAAW0NvbnRlbnRfVHlwZXNdLnhtbG2PSw7CMAxErxJ5n7qwQAg17aJwAy4QBfcjmo8aF4Xbk9AdYunxPM+46ZJdxIvWOHun4FDVIMgZ/5jdqGDjQZ6ha5v7O1AU2eqigok5XBCjmcjqWPlALm8Gv1rNeVxHDNo89Uh4rOsTGu+YHEsuN6BtrjTobWFxS1neYzMOot99JUoBU2IsMv4F7I9dh7DMRnN+ApO0UdoC4rd2+wFQSwECFAAUAAAACACHTuJAf7/Typ0AAADkAAAAEwAAAAAAAAABACAAAABaAQAAW0NvbnRlbnRfVHlwZXNdLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAHAAAAAAAAAAAAEAAAAAAAAABDb25maWcvUEsBAhQAFAAAAAgAh07iQBI4/pifAAAA8wAAABIAAAAAAAAAAQAgAAAAJQAAAENvbmZpZy9QYWNrYWdlLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAAAAAAAAAAEAAAAPQAAABGb3JtdWxhcy9QSwECFAAUAAAACACHTuJAKIpHuA4AAAARAAAAEwAAAAAAAAABACAAAAAbAQAARm9ybXVsYXMvU2VjdGlvbjEubVBLBQYAAAAABQAFAC4BAAAoAgAAAAAOAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PFBlcm1pc3Npb25MaXN0IHhtbG5zOnhzZD0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEiIHhtbG5zOnhzaT0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEtaW5zdGFuY2UiPjxDYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPmZhbHNlPC9DYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPjxGaXJld2FsbEVuYWJsZWQ+dHJ1ZTwvRmlyZXdhbGxFbmFibGVkPjwvUGVybWlzc2lvbkxpc3Q+lQEAAAAAAABzAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PExvY2FsUGFja2FnZU1ldGFkYXRhRmlsZSB4bWxuczp4c2Q9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hIiB4bWxuczp4c2k9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hLWluc3RhbmNlIj48SXRlbXM+PEl0ZW0+PEl0ZW1Mb2NhdGlvbj48SXRlbVR5cGU+QWxsRm9ybXVsYXM8L0l0ZW1UeXBlPjxJdGVtUGF0aCAvPjwvSXRlbUxvY2F0aW9uPjxTdGFibGVFbnRyaWVzPjxFbnRyeSBUeXBlPSJSZWxhdGlvbnNoaXBzIiBWYWx1ZT0ic0FBQUFBQT09IiAvPjwvU3RhYmxlRW50cmllcz48L0l0ZW0+PC9JdGVtcz48L0xvY2FsUGFja2FnZU1ldGFkYXRhRmlsZT4WAAAAUEsFBgAAAAAAAAAAAAAAAAAAAAAAACYBAAABAAAA0Iyd3wEV0RGMegDAT8KX6wEAAAClX4eItUGWQ7NHi8+tDMopAAAAAAIAAAAAABBmAAAAAQAAIAAAAAUeel4tta7v1Hgq64dbhuH1hzmhzLYyWC+BAD8G7y3JAAAAAA6AAAAAAgAAIAAAACyOO8Rzhb6ZXj1dfr3WG/5Udf7cnL5+NY5625QRKJFYUAAAABVYLwQ9UJMAyL9Z1LH1ojmi9HfNByW2Gt5GRcfQIB33A1/pA17ENjU+jF3+3HuG1a1gS4Ge/6O+oMfCHTh3jnZT31yQRdPKXIXr3kk+vCv1QAAAAGmCX78nhkdzRec6RsHFZpbxqLwt7G4y0aw13rdOxk9dvrBqk9rPJ0MzHskra5TbLvMsUmY0uDtKz2R+tf2CStk=</DataMashup>
+<DataMashup xmlns="http://schemas.microsoft.com/DataMashup">AAAAAGwDAABQSwMECgAAAAAAh07iQAAAAAAAAAAAAAAAAAcAAABDb25maWcvUEsDBBQAAAAIAIdO4kASOP6YnwAAAPMAAAASAAAAQ29uZmlnL1BhY2thZ2UueG1shY9NC4IwHMa/iuzuNmdRyN958JoRBNF1zDVHOsPNJn36jDK6dXtefofngWLq2uiuBmd6m6MEUxQpK/vaWJ2j0V/iLSo4HIS8Cq2iGbYum1ydo8b7W0ZICAGHFPeDJozShJyr3VE2qhPoC5v/cGys88JKhTic3mM4w8lqg9N1iimQJYTK2EUzzOa9r/YnhHJs/Tgo/mjicg9ksUA+H/gTUEsDBAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAARm9ybXVsYXMvUEsDBBQAAAAIAIdO4kAoike4DgAAABEAAAATAAAARm9ybXVsYXMvU2VjdGlvbjEubStOTS7JzM9TCIbQhtYAUEsDBBQAAAAIAIdO4kB/v9PKnQAAAOQAAAATAAAAW0NvbnRlbnRfVHlwZXNdLnhtbG2PSw7CMAxErxJ5n7qwQAg17aJwAy4QBfcjmo8aF4Xbk9AdYunxPM+46ZJdxIvWOHun4FDVIMgZ/5jdqGDjQZ6ha5v7O1AU2eqigok5XBCjmcjqWPlALm8Gv1rNeVxHDNo89Uh4rOsTGu+YHEsuN6BtrjTobWFxS1neYzMOot99JUoBU2IsMv4F7I9dh7DMRnN+ApO0UdoC4rd2+wFQSwECFAAUAAAACACHTuJAf7/Typ0AAADkAAAAEwAAAAAAAAABACAAAABaAQAAW0NvbnRlbnRfVHlwZXNdLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAHAAAAAAAAAAAAEAAAAAAAAABDb25maWcvUEsBAhQAFAAAAAgAh07iQBI4/pifAAAA8wAAABIAAAAAAAAAAQAgAAAAJQAAAENvbmZpZy9QYWNrYWdlLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAAAAAAAAAAEAAAAPQAAABGb3JtdWxhcy9QSwECFAAUAAAACACHTuJAKIpHuA4AAAARAAAAEwAAAAAAAAABACAAAAAbAQAARm9ybXVsYXMvU2VjdGlvbjEubVBLBQYAAAAABQAFAC4BAAAoAgAAAAAOAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PFBlcm1pc3Npb25MaXN0IHhtbG5zOnhzZD0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEiIHhtbG5zOnhzaT0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEtaW5zdGFuY2UiPjxDYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPmZhbHNlPC9DYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPjxGaXJld2FsbEVuYWJsZWQ+dHJ1ZTwvRmlyZXdhbGxFbmFibGVkPjwvUGVybWlzc2lvbkxpc3Q+lQEAAAAAAABzAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PExvY2FsUGFja2FnZU1ldGFkYXRhRmlsZSB4bWxuczp4c2Q9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hIiB4bWxuczp4c2k9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hLWluc3RhbmNlIj48SXRlbXM+PEl0ZW0+PEl0ZW1Mb2NhdGlvbj48SXRlbVR5cGU+QWxsRm9ybXVsYXM8L0l0ZW1UeXBlPjxJdGVtUGF0aCAvPjwvSXRlbUxvY2F0aW9uPjxTdGFibGVFbnRyaWVzPjxFbnRyeSBUeXBlPSJSZWxhdGlvbnNoaXBzIiBWYWx1ZT0ic0FBQUFBQT09IiAvPjwvU3RhYmxlRW50cmllcz48L0l0ZW0+PC9JdGVtcz48L0xvY2FsUGFja2FnZU1ldGFkYXRhRmlsZT4WAAAAUEsFBgAAAAAAAAAAAAAAAAAAAAAAACYBAAABAAAA0Iyd3wEV0RGMegDAT8KX6wEAAAClX4eItUGWQ7NHi8+tDMopAAAAAAIAAAAAABBmAAAAAQAAIAAAAIUbDuWLbzOYm1Y2LIS3fNLnp6vuunqZsnJbZYjMjD33AAAAAA6AAAAAAgAAIAAAANpk4QFKMJxrsRq/Rix1uxsd9TnziiMp99XTJvhoNwB9UAAAAOvqWdcsoXOWF9Hdk/e7sfkMs5dcDy1NywO7H8vcRdRvcQoEhncIeVgiz3jmj3r4DkpTyLv1SYQCTObp8Tq4MPbgYH6jniVTh63WhDSMbmWuQAAAAO4xdbs04BtE3lwmIEongvARMYFAr+GkLtKebH0k5D1HxPUZanqfR2F2X6b3Pr89DdpYjSrRAxEVEXlKuj9HYnA=</DataMashup>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC6B7CF5-892E-4D56-AA7F-2137A82D9D20}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53417652-FD3D-443C-86B0-F76B17835802}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
   </ds:schemaRefs>

</xml_diff>